<commit_message>
Segunda versão requisitor pesquisas de referência
Segunda versão da Lista com Requisitos identificado por pesquisas de referência
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
@@ -1,55 +1,201 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guilherme\Downloads\Projetos2SIPG\PastaDocsEngenhariaSw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E0C999-FD68-4061-8901-66FC8701389B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C20E8A-02C5-4C03-BF95-F9C33527B536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>LISTA DE REQUISITOS DO PROJETO DE SISTEMAS DE INFORMAÇÃO PARA GERENCIAR ESTACIONAMENTOS</t>
-  </si>
-  <si>
-    <t>*Legenda: Rf - Requisito Funcional; Rnf - Requisito não funcional</t>
-  </si>
-  <si>
-    <t>id*</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+  <si>
+    <t>LISTA DE REQUISITOS DO PROJETO DE SISTEMA DE INFORMAÇÃO PARA GERENCIAR ESTACIONAMENTOS</t>
+  </si>
+  <si>
+    <t>Id*</t>
   </si>
   <si>
     <t>Nome do requisito</t>
   </si>
   <si>
-    <t>Descrição regra de domínio</t>
+    <t>Descrição da regra de domínio</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*Legenda:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Rf - Requisito funcional; Rnf - Requisito não funcional</t>
+    </r>
+  </si>
+  <si>
+    <t>Rf001</t>
+  </si>
+  <si>
+    <t>Tarifacao inteligente</t>
+  </si>
+  <si>
+    <t>Planos mensais</t>
+  </si>
+  <si>
+    <t>Rf002</t>
+  </si>
+  <si>
+    <t>Parcerias de convênios</t>
+  </si>
+  <si>
+    <t>Rf003</t>
+  </si>
+  <si>
+    <t>Acompanhamento do caixa</t>
+  </si>
+  <si>
+    <t>Rf004</t>
+  </si>
+  <si>
+    <t>Criação de anotações/lembretes</t>
+  </si>
+  <si>
+    <t>Rf005</t>
+  </si>
+  <si>
+    <t>Criação de vouchers de desconto</t>
+  </si>
+  <si>
+    <t>Rf006</t>
+  </si>
+  <si>
+    <t>Controle de serviços extras</t>
+  </si>
+  <si>
+    <t>Acréscimo de serviços como lava-jato, lava-rápido, cera, polimento.</t>
+  </si>
+  <si>
+    <t>Proteção do sistema com anti-fraude</t>
+  </si>
+  <si>
+    <t>Rf007</t>
+  </si>
+  <si>
+    <t>Rf008</t>
+  </si>
+  <si>
+    <t>Localizar estacionamentos disponíveis</t>
+  </si>
+  <si>
+    <t>Rf009</t>
+  </si>
+  <si>
+    <t>Aplicação móvel para motoristas acharem estacionamentos com vagas livres na região em que estão, com seu preços para o horário e dia.</t>
+  </si>
+  <si>
+    <t>Reserva de vaga em tempo real</t>
+  </si>
+  <si>
+    <t>Um motorista em movimento ou antes de sair com seu carro pode reservar uma vaga para um dia e horário em um estacionamento.</t>
+  </si>
+  <si>
+    <t>Rf010</t>
+  </si>
+  <si>
+    <t>Pagamento integrado</t>
+  </si>
+  <si>
+    <t>Aceitar pagamento com cartões ou PIX.</t>
+  </si>
+  <si>
+    <t>Dashboard/painel de acompanhamento de ocupação por mês</t>
+  </si>
+  <si>
+    <t>Apresentar um gráfico de barras com a quantidade de veículos por dia de um mês selecionado.</t>
+  </si>
+  <si>
+    <t>Dashboard/painel de acompanhamento de receitas mês a mês</t>
+  </si>
+  <si>
+    <t>Apresentar um gráfico de linhas com os meses no eixo X e o montante de valor recebido em R$, no eixo Y</t>
+  </si>
+  <si>
+    <t>Rf011</t>
+  </si>
+  <si>
+    <t>Rf012</t>
+  </si>
+  <si>
+    <t>Rf013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notificações de tempo restante </t>
+  </si>
+  <si>
+    <t>Rf014</t>
+  </si>
+  <si>
+    <t>Com auxílio de IA, o sistema vai propor uma tarifa conforme as práticas dos concorrentes na região</t>
+  </si>
+  <si>
+    <t>Tabela de preços exclusiva para mensalistas</t>
+  </si>
+  <si>
+    <t>Tabela de preços exclusiva para conveniados</t>
+  </si>
+  <si>
+    <t>Planos avulsos</t>
+  </si>
+  <si>
+    <t>Tabela de preços exclusiva para estacionamento avulso, cobrado conforme dia e horário</t>
+  </si>
+  <si>
+    <t>Registro de pagamentos com controle fiscal</t>
+  </si>
+  <si>
+    <t>Gerar automaticamente um voucher de desconto conforme o número de horas que o cliente acumulou em um período (desconto parametrizável)</t>
+  </si>
+  <si>
+    <t>Rf015</t>
+  </si>
+  <si>
+    <t>Enviar mensagem por Whatsapp para o motorista, avisando o tempo restante em caso de fechamento do estacionamento</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -57,16 +203,57 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="5" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -89,13 +276,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -159,7 +361,7 @@
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="Yu Gothic Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -194,7 +396,7 @@
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="Yu Gothic"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
@@ -379,105 +581,192 @@
   <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="39.85546875" customWidth="1"/>
-    <col min="3" max="3" width="49.5703125" customWidth="1"/>
+    <col min="2" max="2" width="56" customWidth="1"/>
+    <col min="3" max="3" width="134.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
+      <c r="A9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="C9" s="1"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
+      <c r="A10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
+      <c r="A11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
+      <c r="A12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="C12" s="1"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="A13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+      <c r="A14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+      <c r="A15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+      <c r="A16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="A17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
+      <c r="A18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
+      <c r="A19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
@@ -495,7 +784,467 @@
       <c r="C22" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007544514C3E525041A50FD90CCA057415" ma:contentTypeVersion="31" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="31637ea0daf1112799c414fb7a1c5b78">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b591360b-72bd-45d7-9362-d2d404a7b4f5" xmlns:ns3="e265a0ad-4171-4359-86dd-7b4a7d920c0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="31b507a7e6f7366b3d32c52605501b23" ns2:_="" ns3:_="">
+    <xsd:import namespace="b591360b-72bd-45d7-9362-d2d404a7b4f5"/>
+    <xsd:import namespace="e265a0ad-4171-4359-86dd-7b4a7d920c0e"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:NotebookType" minOccurs="0"/>
+                <xsd:element ref="ns2:FolderType" minOccurs="0"/>
+                <xsd:element ref="ns2:CultureName" minOccurs="0"/>
+                <xsd:element ref="ns2:AppVersion" minOccurs="0"/>
+                <xsd:element ref="ns2:TeamsChannelId" minOccurs="0"/>
+                <xsd:element ref="ns2:Owner" minOccurs="0"/>
+                <xsd:element ref="ns2:Math_Settings" minOccurs="0"/>
+                <xsd:element ref="ns2:DefaultSectionNames" minOccurs="0"/>
+                <xsd:element ref="ns2:Templates" minOccurs="0"/>
+                <xsd:element ref="ns2:Teachers" minOccurs="0"/>
+                <xsd:element ref="ns2:Students" minOccurs="0"/>
+                <xsd:element ref="ns2:Student_Groups" minOccurs="0"/>
+                <xsd:element ref="ns2:Distribution_Groups" minOccurs="0"/>
+                <xsd:element ref="ns2:LMS_Mappings" minOccurs="0"/>
+                <xsd:element ref="ns2:Invited_Teachers" minOccurs="0"/>
+                <xsd:element ref="ns2:Invited_Students" minOccurs="0"/>
+                <xsd:element ref="ns2:Self_Registration_Enabled" minOccurs="0"/>
+                <xsd:element ref="ns2:Has_Teacher_Only_SectionGroup" minOccurs="0"/>
+                <xsd:element ref="ns2:Is_Collaboration_Space_Locked" minOccurs="0"/>
+                <xsd:element ref="ns2:IsNotebookLocked" minOccurs="0"/>
+                <xsd:element ref="ns2:Teams_Channel_Section_Location" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b591360b-72bd-45d7-9362-d2d404a7b4f5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="e2398b20-2c76-408b-9565-673d41e5947a" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="NotebookType" ma:index="18" nillable="true" ma:displayName="Notebook Type" ma:internalName="NotebookType">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="FolderType" ma:index="19" nillable="true" ma:displayName="Folder Type" ma:internalName="FolderType">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="CultureName" ma:index="20" nillable="true" ma:displayName="Culture Name" ma:internalName="CultureName">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="AppVersion" ma:index="21" nillable="true" ma:displayName="App Version" ma:internalName="AppVersion">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TeamsChannelId" ma:index="22" nillable="true" ma:displayName="Teams Channel Id" ma:internalName="TeamsChannelId">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Owner" ma:index="23" nillable="true" ma:displayName="Owner" ma:internalName="Owner">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:User">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="Math_Settings" ma:index="24" nillable="true" ma:displayName="Math Settings" ma:internalName="Math_Settings">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="DefaultSectionNames" ma:index="25" nillable="true" ma:displayName="Default Section Names" ma:internalName="DefaultSectionNames">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Templates" ma:index="26" nillable="true" ma:displayName="Templates" ma:internalName="Templates">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Teachers" ma:index="27" nillable="true" ma:displayName="Teachers" ma:internalName="Teachers">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="Students" ma:index="28" nillable="true" ma:displayName="Students" ma:internalName="Students">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="Student_Groups" ma:index="29" nillable="true" ma:displayName="Student Groups" ma:internalName="Student_Groups">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="Distribution_Groups" ma:index="30" nillable="true" ma:displayName="Distribution Groups" ma:internalName="Distribution_Groups">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="LMS_Mappings" ma:index="31" nillable="true" ma:displayName="LMS Mappings" ma:internalName="LMS_Mappings">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Invited_Teachers" ma:index="32" nillable="true" ma:displayName="Invited Teachers" ma:internalName="Invited_Teachers">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Invited_Students" ma:index="33" nillable="true" ma:displayName="Invited Students" ma:internalName="Invited_Students">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Self_Registration_Enabled" ma:index="34" nillable="true" ma:displayName="Self Registration Enabled" ma:internalName="Self_Registration_Enabled">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Boolean"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Has_Teacher_Only_SectionGroup" ma:index="35" nillable="true" ma:displayName="Has Teacher Only SectionGroup" ma:internalName="Has_Teacher_Only_SectionGroup">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Boolean"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Is_Collaboration_Space_Locked" ma:index="36" nillable="true" ma:displayName="Is Collaboration Space Locked" ma:internalName="Is_Collaboration_Space_Locked">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Boolean"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="IsNotebookLocked" ma:index="37" nillable="true" ma:displayName="Is Notebook Locked" ma:internalName="IsNotebookLocked">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Boolean"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Teams_Channel_Section_Location" ma:index="38" nillable="true" ma:displayName="Teams Channel Section Location" ma:internalName="Teams_Channel_Section_Location">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e265a0ad-4171-4359-86dd-7b4a7d920c0e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c23cd4d2-30d0-41c5-befb-ac1e14ff498f}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e265a0ad-4171-4359-86dd-7b4a7d920c0e">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TeamsChannelId xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Invited_Students xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e265a0ad-4171-4359-86dd-7b4a7d920c0e" xsi:nil="true"/>
+    <Templates xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Has_Teacher_Only_SectionGroup xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <FolderType xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Teams_Channel_Section_Location xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Self_Registration_Enabled xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Teachers xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Teachers>
+    <Distribution_Groups xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <LMS_Mappings xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <CultureName xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <AppVersion xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <DefaultSectionNames xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <NotebookType xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Students xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Students>
+    <Student_Groups xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Student_Groups>
+    <Invited_Teachers xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <IsNotebookLocked xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Is_Collaboration_Space_Locked xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Math_Settings xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Owner xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Owner>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41720870-04A1-40A2-9E0B-C33CEAB5891E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{312D7B65-6127-418F-9F65-8D661FC39729}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8227AD58-3EC3-4518-9BD0-EF16C619881B}"/>
 </file>
</xml_diff>

<commit_message>
3a versao com Brainstorm
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaDeRequisitosSiEstacionamento.xlsx
@@ -1,42 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30002"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C20E8A-02C5-4C03-BF95-F9C33527B536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="13_ncr:1_{51C20E8A-02C5-4C03-BF95-F9C33527B536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9815B63C-EA17-4A66-9B95-8C13D6537D0A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>LISTA DE REQUISITOS DO PROJETO DE SISTEMA DE INFORMAÇÃO PARA GERENCIAR ESTACIONAMENTOS</t>
-  </si>
-  <si>
-    <t>Id*</t>
-  </si>
-  <si>
-    <t>Nome do requisito</t>
-  </si>
-  <si>
-    <t>Descrição da regra de domínio</t>
   </si>
   <si>
     <r>
@@ -62,40 +64,67 @@
     </r>
   </si>
   <si>
+    <t>Id*</t>
+  </si>
+  <si>
+    <t>Nome do requisito</t>
+  </si>
+  <si>
+    <t>Descrição da regra de domínio</t>
+  </si>
+  <si>
     <t>Rf001</t>
   </si>
   <si>
     <t>Tarifacao inteligente</t>
   </si>
   <si>
+    <t>Com auxílio de IA, o sistema vai propor uma tarifa conforme as práticas dos concorrentes na região</t>
+  </si>
+  <si>
+    <t>Rf002</t>
+  </si>
+  <si>
     <t>Planos mensais</t>
   </si>
   <si>
-    <t>Rf002</t>
+    <t>Tabela de preços exclusiva para mensalistas</t>
+  </si>
+  <si>
+    <t>Rf003</t>
   </si>
   <si>
     <t>Parcerias de convênios</t>
   </si>
   <si>
-    <t>Rf003</t>
+    <t>Tabela de preços exclusiva para conveniados</t>
+  </si>
+  <si>
+    <t>Rf004</t>
   </si>
   <si>
     <t>Acompanhamento do caixa</t>
   </si>
   <si>
-    <t>Rf004</t>
+    <t>Registro de pagamentos com controle fiscal</t>
+  </si>
+  <si>
+    <t>Rf005</t>
   </si>
   <si>
     <t>Criação de anotações/lembretes</t>
   </si>
   <si>
-    <t>Rf005</t>
+    <t>Rf006</t>
   </si>
   <si>
     <t>Criação de vouchers de desconto</t>
   </si>
   <si>
-    <t>Rf006</t>
+    <t>Gerar automaticamente um voucher de desconto conforme o número de horas que o cliente acumulou em um período (desconto parametrizável)</t>
+  </si>
+  <si>
+    <t>Rf007</t>
   </si>
   <si>
     <t>Controle de serviços extras</t>
@@ -104,31 +133,34 @@
     <t>Acréscimo de serviços como lava-jato, lava-rápido, cera, polimento.</t>
   </si>
   <si>
+    <t>Rf008</t>
+  </si>
+  <si>
     <t>Proteção do sistema com anti-fraude</t>
   </si>
   <si>
-    <t>Rf007</t>
-  </si>
-  <si>
-    <t>Rf008</t>
+    <t>Controle por câmeras LPR: Automação total e antifraude completo com câmeras de leitura de placa</t>
+  </si>
+  <si>
+    <t>Rf009</t>
   </si>
   <si>
     <t>Localizar estacionamentos disponíveis</t>
   </si>
   <si>
-    <t>Rf009</t>
-  </si>
-  <si>
     <t>Aplicação móvel para motoristas acharem estacionamentos com vagas livres na região em que estão, com seu preços para o horário e dia.</t>
   </si>
   <si>
+    <t>Rf010</t>
+  </si>
+  <si>
     <t>Reserva de vaga em tempo real</t>
   </si>
   <si>
     <t>Um motorista em movimento ou antes de sair com seu carro pode reservar uma vaga para um dia e horário em um estacionamento.</t>
   </si>
   <si>
-    <t>Rf010</t>
+    <t>Rf011</t>
   </si>
   <si>
     <t>Pagamento integrado</t>
@@ -137,40 +169,34 @@
     <t>Aceitar pagamento com cartões ou PIX.</t>
   </si>
   <si>
+    <t>Rf012</t>
+  </si>
+  <si>
     <t>Dashboard/painel de acompanhamento de ocupação por mês</t>
   </si>
   <si>
     <t>Apresentar um gráfico de barras com a quantidade de veículos por dia de um mês selecionado.</t>
   </si>
   <si>
+    <t>Rf013</t>
+  </si>
+  <si>
     <t>Dashboard/painel de acompanhamento de receitas mês a mês</t>
   </si>
   <si>
     <t>Apresentar um gráfico de linhas com os meses no eixo X e o montante de valor recebido em R$, no eixo Y</t>
   </si>
   <si>
-    <t>Rf011</t>
-  </si>
-  <si>
-    <t>Rf012</t>
-  </si>
-  <si>
-    <t>Rf013</t>
+    <t>Rf014</t>
   </si>
   <si>
     <t xml:space="preserve">Notificações de tempo restante </t>
   </si>
   <si>
-    <t>Rf014</t>
-  </si>
-  <si>
-    <t>Com auxílio de IA, o sistema vai propor uma tarifa conforme as práticas dos concorrentes na região</t>
-  </si>
-  <si>
-    <t>Tabela de preços exclusiva para mensalistas</t>
-  </si>
-  <si>
-    <t>Tabela de preços exclusiva para conveniados</t>
+    <t>Enviar mensagem por Whatsapp para o motorista, avisando o tempo restante em caso de fechamento do estacionamento</t>
+  </si>
+  <si>
+    <t>Rf015</t>
   </si>
   <si>
     <t>Planos avulsos</t>
@@ -179,23 +205,107 @@
     <t>Tabela de preços exclusiva para estacionamento avulso, cobrado conforme dia e horário</t>
   </si>
   <si>
-    <t>Registro de pagamentos com controle fiscal</t>
-  </si>
-  <si>
-    <t>Gerar automaticamente um voucher de desconto conforme o número de horas que o cliente acumulou em um período (desconto parametrizável)</t>
-  </si>
-  <si>
-    <t>Rf015</t>
-  </si>
-  <si>
-    <t>Enviar mensagem por Whatsapp para o motorista, avisando o tempo restante em caso de fechamento do estacionamento</t>
+    <t>Rf016</t>
+  </si>
+  <si>
+    <t>Historico de clientes</t>
+  </si>
+  <si>
+    <t>Armazenar dados de clientes frequentes como placa, horários utilizados e serviços extras utilizados.</t>
+  </si>
+  <si>
+    <t>Rf017</t>
+  </si>
+  <si>
+    <t>Gestão de vagas especiais</t>
+  </si>
+  <si>
+    <t>O sistema deve permitir a configuração de vagas exclusivas (idosos, PCD, elétricos).</t>
+  </si>
+  <si>
+    <t>Rf018</t>
+  </si>
+  <si>
+    <t>Sistema de Senhas</t>
+  </si>
+  <si>
+    <t>Rf019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestão de assinaturas corporativas </t>
+  </si>
+  <si>
+    <t>empresas podem comprar pacotes de vagas e gerenciar permissões dos funcionários.</t>
+  </si>
+  <si>
+    <t>Rf020</t>
+  </si>
+  <si>
+    <t>Sistema de avaliação de clientes</t>
+  </si>
+  <si>
+    <t>Clientes podem avaliar o estacionamento e deixar feedback sobre segurança, limpeza e atendimento.</t>
+  </si>
+  <si>
+    <t>Rf021</t>
+  </si>
+  <si>
+    <t>Relatório de horários de pico</t>
+  </si>
+  <si>
+    <t>O sistema analisa os horários com maior quantidade de veículos para ajudar na gestão do estacionamento.</t>
+  </si>
+  <si>
+    <t>Rf022</t>
+  </si>
+  <si>
+    <t>Relatorio de ocupaçãopor horário/dia</t>
+  </si>
+  <si>
+    <t>Demonstração de horarios de pico</t>
+  </si>
+  <si>
+    <t>Rf023</t>
+  </si>
+  <si>
+    <t>Controle de fila de espera</t>
+  </si>
+  <si>
+    <t>O sistema deve gerenciar uma fila virtual quando não houver vagas disponíveis.</t>
+  </si>
+  <si>
+    <t>Rf024</t>
+  </si>
+  <si>
+    <t>Integração com cancela automática</t>
+  </si>
+  <si>
+    <t>Controlar a abertura e fechamento de cancelas na entrada e saída (entrada após emissão do ticket e saída após pagamento)</t>
+  </si>
+  <si>
+    <t>Rnf001</t>
+  </si>
+  <si>
+    <t>Padrão de tela</t>
+  </si>
+  <si>
+    <t>Tela com fundo azul marinho e letras em branco</t>
+  </si>
+  <si>
+    <t>Rnf002</t>
+  </si>
+  <si>
+    <t>Identificação do estacionamento usuário do sistema</t>
+  </si>
+  <si>
+    <t>Colocar o Logo da nossa empresa de software, no alto, do lado direito da tela e o logo do estacionamento no alto, do lado esquerdo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -253,7 +363,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -287,17 +397,84 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -578,36 +755,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="56" customWidth="1"/>
     <col min="3" max="3" width="134.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -615,173 +792,287 @@
         <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="1"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="10"/>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B26" t="s">
+        <v>67</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="8"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -790,6 +1081,71 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TeamsChannelId xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Invited_Students xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e265a0ad-4171-4359-86dd-7b4a7d920c0e" xsi:nil="true"/>
+    <Templates xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Has_Teacher_Only_SectionGroup xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <FolderType xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Teams_Channel_Section_Location xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Self_Registration_Enabled xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Teachers xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Teachers>
+    <Distribution_Groups xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <LMS_Mappings xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <CultureName xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <AppVersion xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <DefaultSectionNames xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <NotebookType xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Students xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Students>
+    <Student_Groups xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Student_Groups>
+    <Invited_Teachers xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <IsNotebookLocked xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Is_Collaboration_Space_Locked xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <Math_Settings xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Owner xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Owner>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007544514C3E525041A50FD90CCA057415" ma:contentTypeVersion="31" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="31637ea0daf1112799c414fb7a1c5b78">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b591360b-72bd-45d7-9362-d2d404a7b4f5" xmlns:ns3="e265a0ad-4171-4359-86dd-7b4a7d920c0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="31b507a7e6f7366b3d32c52605501b23" ns2:_="" ns3:_="">
     <xsd:import namespace="b591360b-72bd-45d7-9362-d2d404a7b4f5"/>
@@ -1172,73 +1528,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TeamsChannelId xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <Invited_Students xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e265a0ad-4171-4359-86dd-7b4a7d920c0e" xsi:nil="true"/>
-    <Templates xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <Has_Teacher_Only_SectionGroup xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <FolderType xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <Teams_Channel_Section_Location xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <Self_Registration_Enabled xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <Teachers xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Teachers>
-    <Distribution_Groups xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <LMS_Mappings xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <CultureName xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <AppVersion xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <DefaultSectionNames xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <NotebookType xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <Students xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Students>
-    <Student_Groups xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Student_Groups>
-    <Invited_Teachers xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <IsNotebookLocked xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <Is_Collaboration_Space_Locked xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <Math_Settings xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Owner xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Owner>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41720870-04A1-40A2-9E0B-C33CEAB5891E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8227AD58-3EC3-4518-9BD0-EF16C619881B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1246,5 +1537,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8227AD58-3EC3-4518-9BD0-EF16C619881B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41720870-04A1-40A2-9E0B-C33CEAB5891E}"/>
 </file>
</xml_diff>